<commit_message>
commit 20/04/26 a Mac
</commit_message>
<xml_diff>
--- a/CYP2B6/CYP2B6_Allele_def_rs_excluidos.xlsx
+++ b/CYP2B6/CYP2B6_Allele_def_rs_excluidos.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23010" windowHeight="9015" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25200" windowHeight="11160" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Salida_R" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="258" uniqueCount="97">
   <si>
     <t>rsID</t>
   </si>
@@ -301,7 +301,16 @@
     <t>Corresponde al rs2516199080 (CYP2B6_allele_definition_table)</t>
   </si>
   <si>
-    <t xml:space="preserve">dbSNP, genomAD, UCSC </t>
+    <t>https://www.clinpgx.org/haplotype/PA165818811</t>
+  </si>
+  <si>
+    <t>CYP2B6_frequency_table</t>
+  </si>
+  <si>
+    <t>https://www.clinpgx.org/haplotype/PA165818813</t>
+  </si>
+  <si>
+    <t>https://www.clinpgx.org/haplotype/PA166117272</t>
   </si>
 </sst>
 </file>
@@ -336,7 +345,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -364,12 +373,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF00B0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF7030A0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -402,7 +405,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -425,9 +428,7 @@
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -1342,7 +1343,9 @@
       <c r="Y4" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="Z4" s="7"/>
+      <c r="Z4" s="7" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
@@ -1363,7 +1366,9 @@
       <c r="Y5" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="Z5" s="7"/>
+      <c r="Z5" s="7" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
@@ -1384,7 +1389,9 @@
       <c r="Y6" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="Z6" s="7"/>
+      <c r="Z6" s="7" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
@@ -1396,16 +1403,22 @@
       <c r="T7" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="U7" s="14"/>
-      <c r="V7" s="15" t="s">
+      <c r="U7" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="V7" s="14" t="s">
         <v>92</v>
       </c>
-      <c r="W7" s="16"/>
+      <c r="W7" s="8">
+        <v>0</v>
+      </c>
       <c r="X7" s="7"/>
       <c r="Y7" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z7" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="Z7" s="7"/>
     </row>
     <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
@@ -1417,12 +1430,20 @@
       <c r="T8" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="U8" s="8"/>
+      <c r="U8" s="9" t="s">
+        <v>51</v>
+      </c>
       <c r="V8" s="8"/>
-      <c r="W8" s="7"/>
+      <c r="W8" s="7">
+        <v>0</v>
+      </c>
       <c r="X8" s="7"/>
-      <c r="Y8" s="7"/>
-      <c r="Z8" s="7"/>
+      <c r="Y8" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z8" s="7" t="s">
+        <v>95</v>
+      </c>
     </row>
     <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
@@ -1434,12 +1455,20 @@
       <c r="T9" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="U9" s="8"/>
+      <c r="U9" s="9" t="s">
+        <v>53</v>
+      </c>
       <c r="V9" s="8"/>
-      <c r="W9" s="7"/>
+      <c r="W9" s="7">
+        <v>0</v>
+      </c>
       <c r="X9" s="7"/>
-      <c r="Y9" s="7"/>
-      <c r="Z9" s="7"/>
+      <c r="Y9" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="Z9" s="7" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
@@ -1460,7 +1489,9 @@
       <c r="Y10" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="Z10" s="7"/>
+      <c r="Z10" s="7" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
@@ -1481,7 +1512,9 @@
       <c r="Y11" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="Z11" s="7"/>
+      <c r="Z11" s="7" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">

</xml_diff>